<commit_message>
Fixed the total area of Denmark
</commit_message>
<xml_diff>
--- a/area_tbl.xlsx
+++ b/area_tbl.xlsx
@@ -380,10 +380,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>1596.3811301323</v>
+        <v>1596.38113013229</v>
       </c>
       <c r="C2" t="n">
-        <v>3.70012314605113</v>
+        <v>3.70005040544428</v>
       </c>
     </row>
     <row r="3">
@@ -394,7 +394,7 @@
         <v>36298.1396261912</v>
       </c>
       <c r="C3" t="n">
-        <v>84.1325320466141</v>
+        <v>84.1308780877608</v>
       </c>
     </row>
     <row r="4">
@@ -405,7 +405,7 @@
         <v>2026.65606284671</v>
       </c>
       <c r="C4" t="n">
-        <v>4.69742273049952</v>
+        <v>4.69733038401091</v>
       </c>
     </row>
     <row r="5">
@@ -416,7 +416,7 @@
         <v>736.644195626221</v>
       </c>
       <c r="C5" t="n">
-        <v>1.70740820421431</v>
+        <v>1.70737463832907</v>
       </c>
     </row>
     <row r="6">
@@ -427,7 +427,7 @@
         <v>2529.90342608951</v>
       </c>
       <c r="C6" t="n">
-        <v>5.86385922976431</v>
+        <v>5.86374395233652</v>
       </c>
     </row>
   </sheetData>

</xml_diff>